<commit_message>
Principal role uer 504
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0037504_VerifyTheTASDNDFunctionalityforFVAOpportunityAndEngagementOnSFLightningView.xlsx
+++ b/TestData/LV_TMTT0037504_VerifyTheTASDNDFunctionalityforFVAOpportunityAndEngagementOnSFLightningView.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E663A94B-2650-491E-B028-1BC22C47AD8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10EA8D1-DF20-4F28-856C-8F9E568011F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUser" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="121">
   <si>
     <t>User</t>
   </si>
@@ -405,6 +405,9 @@
   </si>
   <si>
     <t>Blaise Brunda</t>
+  </si>
+  <si>
+    <t>Amy Xia</t>
   </si>
 </sst>
 </file>
@@ -1705,7 +1708,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C57A28D-BDAE-4AE1-A126-325DE86B36F7}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
@@ -1716,7 +1719,7 @@
     <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>103</v>
       </c>
@@ -1736,7 +1739,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>111</v>
       </c>
@@ -1753,9 +1756,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -1771,6 +1774,9 @@
       </c>
       <c r="F3" t="s">
         <v>118</v>
+      </c>
+      <c r="G3" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>